<commit_message>
Marca os hospitais de direcionamento interno com (D)
Erastinho, Erasto Gaertner e Pequeno Principe nao aparecem na busca do 400
nem do CIM, e o Novaclinica nao aparece no CIM - mas os quatro atendem por
encaminhamento da operadora. Antes a tabela mostrava "-" nessas casas, o que
dizia ao cliente que o hospital nao existia naquele plano.

- dados/direcionamento.json: curadoria do corretor, por CNPJ e por plano.
  E o unico arquivo editado a mao; tem _leia_me e esta no README.
- o prestador passa a constar no plano, com D no lugar do visto - na pagina,
  nas planilhas, no comparativo HTML e nos dois PDFs
- legenda em todos: "atende, mas por encaminhamento, nao por acesso livre"
- no 600 os quatro sao rede direta, entao continuam com visto

De quebra, as planilhas ainda usavam a paleta antiga (verde/azul do material
da Amil) nos cabecalhos; agora usam a mesma da pagina e dos PDFs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02 - COMPARATIVOS DE REDE/COMPARATIVO REDE PARANA CLINICAS.xlsx
+++ b/02 - COMPARATIVOS DE REDE/COMPARATIVO REDE PARANA CLINICAS.xlsx
@@ -43,17 +43,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F6B4E"/>
+      <color rgb="006B3F8F"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="002A2ABF"/>
+      <color rgb="00B5761B"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0010233F"/>
+      <color rgb="008E0E28"/>
       <sz val="13"/>
     </font>
     <font>
@@ -69,7 +69,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0010233F"/>
+        <fgColor rgb="008E0E28"/>
       </patternFill>
     </fill>
     <fill>
@@ -79,27 +79,27 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F6B4E"/>
+        <fgColor rgb="006B3F8F"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002A2ABF"/>
+        <fgColor rgb="00B5761B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBEEF1"/>
+        <fgColor rgb="00FDF2F5"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDF5F1"/>
+        <fgColor rgb="00F5F1FA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EEEEFB"/>
+        <fgColor rgb="00FDF6EC"/>
       </patternFill>
     </fill>
   </fills>
@@ -626,17 +626,17 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL SANTA CRUZ</t>
+          <t>HOSPITAL ERASTO GAERTNER</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>76555069000143</t>
+          <t>76591049000128</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>Pronto Socorro, Pronto Socorro Cardiologia, Pronto Socorro Clínica Geral, Pronto Socorro Ginecologia, Pronto Socorro Neurologia, Pronto Socorro Obstetrícia, Pronto Socorro Ortopedia, Pronto Socorro Pediatria, Radiodiagnóstico, Ressonância Magnética, Tomografia Computadorizada</t>
+          <t>Hematologia, Hemoterapia, Pronto Socorro Oncológico</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -646,32 +646,28 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Batel</t>
+          <t>Jardim das Américas</t>
         </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>Avenida Do Batel, 1889</t>
+          <t>Rua Dr. Ovande do Amaral, 201</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>80420-090</t>
+          <t>81520-060</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>(41) 3003-3230</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>relacionamento.rededor@dorconsultoria.com.br</t>
-        </is>
-      </c>
+          <t>(41) 3361-5000</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr"/>
       <c r="L2" s="6" t="inlineStr">
         <is>
-          <t>✔</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M2" s="7" t="inlineStr">
@@ -681,7 +677,7 @@
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
-          <t>✔</t>
+          <t>D</t>
         </is>
       </c>
     </row>
@@ -698,45 +694,49 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL ANGELINA CARON</t>
+          <t>HOSPITAL SANTA CRUZ</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>07088017000191</t>
+          <t>76555069000143</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>Anatomia Patológica e Citopatologia, Cardiologia, Cirurgia Geral, Cirurgia Pediátrica, Clínica Geral, Dermatologia, Endocrinologia e Metabologia, Endoscopia Digestiva, Exames Cardiológicos, Gastroenterologia Pediátrica, Ginecologia, Nefrologia, Nefrologia Pediátrica, Neurocirurgia, Obstetrícia, Oftalmologia, Ortopedia e Traumatologia, Otorrinolaringologia, Pediatria, Pneumologia Pediátrica, Pronto Socorro, Pronto Socorro Obstetrícia, Pronto Socorro Pediatria, Radiodiagnóstico, Radioterapia, Ultrassonografia, Urologia</t>
+          <t>Pronto Socorro, Pronto Socorro Cardiologia, Pronto Socorro Clínica Geral, Pronto Socorro Ginecologia, Pronto Socorro Neurologia, Pronto Socorro Obstetrícia, Pronto Socorro Ortopedia, Pronto Socorro Pediatria, Radiodiagnóstico, Ressonância Magnética, Tomografia Computadorizada</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Campina Grande do Sul</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Araçatuba</t>
+          <t>Batel</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Rodovia Caqui, 1150, Km 01</t>
+          <t>Avenida Do Batel, 1889</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>83430-000</t>
+          <t>80420-090</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>(41) 3679-8100</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr"/>
+          <t>(41) 3003-3230</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>relacionamento.rededor@dorconsultoria.com.br</t>
+        </is>
+      </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -766,49 +766,45 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL DO CENTRO</t>
+          <t>HOSPITAL ANGELINA CARON</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>08689079000111</t>
+          <t>07088017000191</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Pronto Socorro Clínica Geral</t>
+          <t>Anatomia Patológica e Citopatologia, Cardiologia, Cirurgia Geral, Cirurgia Pediátrica, Clínica Geral, Dermatologia, Endocrinologia e Metabologia, Endoscopia Digestiva, Exames Cardiológicos, Gastroenterologia Pediátrica, Ginecologia, Nefrologia, Nefrologia Pediátrica, Neurocirurgia, Obstetrícia, Oftalmologia, Ortopedia e Traumatologia, Otorrinolaringologia, Pediatria, Pneumologia Pediátrica, Pronto Socorro, Pronto Socorro Obstetrícia, Pronto Socorro Pediatria, Radiodiagnóstico, Radioterapia, Ultrassonografia, Urologia</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Campo Largo</t>
+          <t>Campina Grande do Sul</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Centro</t>
+          <t>Araçatuba</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Rua Rocha Pombo, 1064, 3054-7818 Atend. SUS / (41) 3054-7819  Atend. CONV</t>
+          <t>Rodovia Caqui, 1150, Km 01</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>83601-350</t>
+          <t>83430-000</t>
         </is>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
-          <t>(41) 3054-7818</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>comercial@hospitaldorocio.com.br</t>
-        </is>
-      </c>
+          <t>(41) 3679-8100</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -838,17 +834,17 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>MATERNIDADE E CIRURGIA NOSSA SENHORA DO ROCIO</t>
+          <t>HOSPITAL DO CENTRO</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>75802348000100</t>
+          <t>08689079000111</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Anestesiologia, Buco Maxilo Facial, Cardiologia, Cirurgia Geral, Cirurgia Vascular, Endocrinologia e Metabologia, Nefrologia, Neurocirurgia, Oncologia, Ortopedia e Traumatologia, Pronto Socorro</t>
+          <t>Pronto Socorro Clínica Geral</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
@@ -858,27 +854,27 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>São Jeronimo</t>
+          <t>Centro</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Rua Maria Aparecida de Oliveira, 599</t>
+          <t>Rua Rocha Pombo, 1064, 3054-7818 Atend. SUS / (41) 3054-7819  Atend. CONV</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>83601-000</t>
+          <t>83601-350</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>(41) 3136-2515</t>
+          <t>(41) 3054-7818</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>convenios@hospitaldorocio.com.br</t>
+          <t>comercial@hospitaldorocio.com.br</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -910,47 +906,47 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL E MATERNIDADE PINHAIS</t>
+          <t>MATERNIDADE E CIRURGIA NOSSA SENHORA DO ROCIO</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>04803609000150</t>
+          <t>75802348000100</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Clínica Geral, Pronto Socorro, Pronto Socorro Clínica Geral, Pronto Socorro Obstetrícia</t>
+          <t>Anestesiologia, Buco Maxilo Facial, Cardiologia, Cirurgia Geral, Cirurgia Vascular, Endocrinologia e Metabologia, Nefrologia, Neurocirurgia, Oncologia, Ortopedia e Traumatologia, Pronto Socorro</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Pinhais</t>
+          <t>Campo Largo</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Jardim Guaraicá</t>
+          <t>São Jeronimo</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Avenida Jacob Macanhan, 93</t>
+          <t>Rua Maria Aparecida de Oliveira, 599</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>83326-000</t>
+          <t>83601-000</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>(41) 3661-1600</t>
+          <t>(41) 3136-2515</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>faturamentohmp@yahoo.com,</t>
+          <t>convenios@hospitaldorocio.com.br</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -982,47 +978,47 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Hospital Cruz Vermelha Curitiba</t>
+          <t>HOSPITAL E MATERNIDADE PINHAIS</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>07404052000172</t>
+          <t>04803609000150</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Pronto Socorro</t>
+          <t>Clínica Geral, Pronto Socorro, Pronto Socorro Clínica Geral, Pronto Socorro Obstetrícia</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>Curitiba</t>
+          <t>Pinhais</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Batel</t>
+          <t>Jardim Guaraicá</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Avenida Vicente Machado, 1310</t>
+          <t>Avenida Jacob Macanhan, 93</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>80420-011</t>
+          <t>83326-000</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>(41) 3016-6622</t>
+          <t>(41) 3661-1600</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>contratos@cruzvermelhapr.com.br</t>
+          <t>faturamentohmp@yahoo.com,</t>
         </is>
       </c>
       <c r="L7" s="6" t="inlineStr">
@@ -1035,7 +1031,11 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="N7" s="8" t="inlineStr"/>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1050,12 +1050,12 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL DAS NAÇÕES</t>
+          <t>NOVACLÍNICA HOSPITAL E MATERNIDADE</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>77799823000153</t>
+          <t>81306136000126</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1065,32 +1065,32 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Curitiba</t>
+          <t>São José dos Pinhais</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Jardim Social</t>
+          <t>Centro</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Rua Raphael Papa, 10</t>
+          <t>Rua Quinze de Novembro, 2316</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>82530-190</t>
+          <t>83005-000</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>(41) 3306-9000</t>
+          <t>(41) 3381-8100</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr">
         <is>
-          <t>faturamento@hospitalnacoes.com.br</t>
+          <t>faturamento@hnovaclinica.com.br</t>
         </is>
       </c>
       <c r="L8" s="6" t="inlineStr">
@@ -1103,7 +1103,11 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="N8" s="8" t="inlineStr"/>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1118,17 +1122,17 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL UNIVERSITÁRIO EVANGELICO MACKENZIE</t>
+          <t>Hospital Cruz Vermelha Curitiba</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>60967551002102</t>
+          <t>07404052000172</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Cirurgia Geral, Cirurgia Plástica, Clínica Geral, Obstetrícia, Ortopedia e Traumatologia, Pediatria, Pronto Socorro Queimados, Queimados</t>
+          <t>Pronto Socorro</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -1138,25 +1142,29 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Bigorrilho</t>
+          <t>Batel</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Alameda Augusto Stellfeld, 1908</t>
+          <t>Avenida Vicente Machado, 1310</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>80730-150</t>
+          <t>80420-011</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>(41) 3240-5000</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr"/>
+          <t>(41) 3016-6622</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>contratos@cruzvermelhapr.com.br</t>
+        </is>
+      </c>
       <c r="L9" s="6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -1182,45 +1190,49 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL SAO LUCAS</t>
+          <t>HOSPITAL DAS NAÇÕES</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>52695456000117</t>
+          <t>77799823000153</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>Análises Clínicas, Anestesiologia, Cardiologia, Clínica Geral, Ginecologia, Obstetrícia, Oncologia, Ortopedia e Traumatologia, Patologia Clínica/Medicina Laboratorial, Pediatria, Pronto Socorro</t>
+          <t>Pronto Socorro</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Campo Largo</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Centro</t>
+          <t>Jardim Social</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Rua Generoso Marques, 2022</t>
+          <t>Rua Raphael Papa, 10</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>83601-050</t>
+          <t>82530-190</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>(41) 3032-9300</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr"/>
+          <t>(41) 3306-9000</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>faturamento@hospitalnacoes.com.br</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -1246,49 +1258,45 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>NOVACLÍNICA HOSPITAL E MATERNIDADE</t>
+          <t>HOSPITAL UNIVERSITÁRIO EVANGELICO MACKENZIE</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>81306136000126</t>
+          <t>60967551002102</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Pronto Socorro</t>
+          <t>Cirurgia Geral, Cirurgia Plástica, Clínica Geral, Obstetrícia, Ortopedia e Traumatologia, Pediatria, Pronto Socorro Queimados, Queimados</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>São José dos Pinhais</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Centro</t>
+          <t>Bigorrilho</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Rua Quinze de Novembro, 2316</t>
+          <t>Alameda Augusto Stellfeld, 1908</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>83005-000</t>
+          <t>80730-150</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>(41) 3381-8100</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>faturamento@hnovaclinica.com.br</t>
-        </is>
-      </c>
+          <t>(41) 3240-5000</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -1314,46 +1322,50 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL ERASTO GAERTNER</t>
+          <t>HOSPITAL SAO LUCAS</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>76591049000128</t>
+          <t>52695456000117</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Hematologia, Hemoterapia, Pronto Socorro Oncológico</t>
+          <t>Análises Clínicas, Anestesiologia, Cardiologia, Clínica Geral, Ginecologia, Obstetrícia, Oncologia, Ortopedia e Traumatologia, Patologia Clínica/Medicina Laboratorial, Pediatria, Pronto Socorro</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Curitiba</t>
+          <t>Campo Largo</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Jardim das Américas</t>
+          <t>Centro</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Rua Dr. Ovande do Amaral, 201</t>
+          <t>Rua Generoso Marques, 2022</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>81520-060</t>
+          <t>83601-050</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>(41) 3361-5000</t>
+          <t>(41) 3032-9300</t>
         </is>
       </c>
       <c r="K12" s="5" t="inlineStr"/>
-      <c r="L12" s="6" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
           <t>✔</t>
@@ -1758,17 +1770,17 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>OFTALMO CURITIBA - HOSPITAL DA VISAO</t>
+          <t>HOSPITAL ERASTINHO</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>80764889000112</t>
+          <t>76591049000985</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Oftalmologia, Pronto Socorro Oftalmológico</t>
+          <t>Oncologia, Oncologia Pediatrica, Pediatria, Pronto Socorro Oncológico</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
@@ -1778,32 +1790,28 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Batel</t>
+          <t>Jardim das Américas</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Rua Bispo Dom José, 2711</t>
+          <t>Rua Doutor Ovande do Amaral, 201</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>80440-080</t>
+          <t>81520-060</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>(41) 3016-4030</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>oftalmologia@oftalmocuritiba.com.br</t>
-        </is>
-      </c>
+          <t>(41) 3165-4504</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr"/>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>✔</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M19" s="7" t="inlineStr">
@@ -1813,7 +1821,7 @@
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>✔</t>
+          <t>D</t>
         </is>
       </c>
     </row>
@@ -1830,52 +1838,48 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>CADMO CLINICA PSIQUIATRICA</t>
+          <t>HOSPITAL INFANTIL PEQUENO PRINCIPE</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>05343133000184</t>
+          <t>76591569000130</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>Psiquiatria, Psiquiatria da Infância e Adolescência</t>
+          <t>Cirurgia Pediátrica, Dermatologia Pediátrica, Neurologia Pediátrica, Oncologia, Otorrinolaringologia, Pediatria, Pronto Socorro Pediatria, Reumatologia Infantil</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Piraquara</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Cayva</t>
+          <t>Água Verde</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Rua José Erasmo Storniolo, 450, Telefone: 0800 323 5088</t>
+          <t>Rua Desembargador Motta, 1070</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>83304-450</t>
+          <t>80250-060</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>(08) 00323-5088</t>
-        </is>
-      </c>
-      <c r="K20" s="5" t="inlineStr">
-        <is>
-          <t>alicia.santos@vivsaude.com.br</t>
-        </is>
-      </c>
+          <t>(41) 3310-1010</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr"/>
       <c r="L20" s="6" t="inlineStr">
         <is>
-          <t>✔</t>
+          <t>D</t>
         </is>
       </c>
       <c r="M20" s="7" t="inlineStr">
@@ -1885,7 +1889,7 @@
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>✔</t>
+          <t>D</t>
         </is>
       </c>
     </row>
@@ -1902,17 +1906,17 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>CDOP Cirurgia Diagnose em Oftalmologia Pr</t>
+          <t>OFTALMO CURITIBA - HOSPITAL DA VISAO</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>00395490000172</t>
+          <t>80764889000112</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Oftalmologia</t>
+          <t>Oftalmologia, Pronto Socorro Oftalmológico</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1922,27 +1926,27 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Seminário</t>
+          <t>Batel</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Avenida Silva Jardim, 4172</t>
+          <t>Rua Bispo Dom José, 2711</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>80240-021</t>
+          <t>80440-080</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>(41) 3221-3600</t>
+          <t>(41) 3016-4030</t>
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr">
         <is>
-          <t>supervisao.atendimento@cdop.com.br</t>
+          <t>oftalmologia@oftalmocuritiba.com.br</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
@@ -1955,7 +1959,11 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="N21" s="8" t="inlineStr"/>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1970,45 +1978,49 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL E MATERNIDADE SANTA BRIGIDA</t>
+          <t>CADMO CLINICA PSIQUIATRICA</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>76882612006158</t>
+          <t>05343133000184</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Ginecologia, Obstetrícia, Pronto Socorro Obstetrícia</t>
+          <t>Psiquiatria, Psiquiatria da Infância e Adolescência</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>Curitiba</t>
+          <t>Piraquara</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Água Verde</t>
+          <t>Cayva</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Rua Guilherme Pugsley, 1705</t>
+          <t>Rua José Erasmo Storniolo, 450, Telefone: 0800 323 5088</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>80620-000</t>
+          <t>83304-450</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>(41) 3232-2500</t>
-        </is>
-      </c>
-      <c r="K22" s="5" t="inlineStr"/>
+          <t>(08) 00323-5088</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr">
+        <is>
+          <t>alicia.santos@vivsaude.com.br</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -2019,7 +2031,11 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="N22" s="8" t="inlineStr"/>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2034,17 +2050,17 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Hospital XV</t>
+          <t>CDOP Cirurgia Diagnose em Oftalmologia Pr</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>76530518000107</t>
+          <t>00395490000172</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Pronto Socorro Ortopedia</t>
+          <t>Oftalmologia</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -2054,25 +2070,29 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Alto da Rua XV</t>
+          <t>Seminário</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Rua XV de Novembro, 2223</t>
+          <t>Avenida Silva Jardim, 4172</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>80045-125</t>
+          <t>80240-021</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>(41) 3218-2000</t>
-        </is>
-      </c>
-      <c r="K23" s="5" t="inlineStr"/>
+          <t>(41) 3221-3600</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>supervisao.atendimento@cdop.com.br</t>
+        </is>
+      </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
           <t>✔</t>
@@ -2098,42 +2118,42 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>OFTALMO CURITIBA - HOSPITAL DA VISAO</t>
+          <t>HOSPITAL E MATERNIDADE SANTA BRIGIDA</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>80764889000112</t>
+          <t>76882612006158</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>Oftalmologia</t>
+          <t>Ginecologia, Obstetrícia, Pronto Socorro Obstetrícia</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>São José dos Pinhais</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Centro</t>
+          <t>Água Verde</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Rua Voluntários da Pátria, 300</t>
+          <t>Rua Guilherme Pugsley, 1705</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>80005-430</t>
+          <t>80620-000</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>(41) 3340-3030</t>
+          <t>(41) 3232-2500</t>
         </is>
       </c>
       <c r="K24" s="5" t="inlineStr"/>
@@ -2142,12 +2162,12 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="M24" s="7" t="inlineStr"/>
-      <c r="N24" s="8" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
+      <c r="M24" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="N24" s="8" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2162,42 +2182,42 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>OFTALMO CURITIBA - HOSPITAL DA VISAO</t>
+          <t>Hospital XV</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>80764889000112</t>
+          <t>76530518000107</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Oftalmologia</t>
+          <t>Pronto Socorro Ortopedia</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>São José dos Pinhais</t>
+          <t>Curitiba</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>São Pedro</t>
+          <t>Alto da Rua XV</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Rua Alcídio Viana, 1001, 5º andar consultório 53 exames sala 51e 52</t>
+          <t>Rua XV de Novembro, 2223</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>83005-560</t>
+          <t>80045-125</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>(41) 3146-1566</t>
+          <t>(41) 3218-2000</t>
         </is>
       </c>
       <c r="K25" s="5" t="inlineStr"/>
@@ -2206,12 +2226,12 @@
           <t>✔</t>
         </is>
       </c>
-      <c r="M25" s="7" t="inlineStr"/>
-      <c r="N25" s="8" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
+      <c r="M25" s="7" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="N25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -2226,56 +2246,56 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>ARTRO CLINICA ORTOPEDICA</t>
+          <t>OFTALMO CURITIBA - HOSPITAL DA VISAO</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>11402669000126</t>
+          <t>80764889000112</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Ortopedia e Traumatologia</t>
+          <t>Oftalmologia</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Curitiba</t>
+          <t>São José dos Pinhais</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Batel</t>
+          <t>Centro</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Avenida Vicente Machado, 2411</t>
+          <t>Rua Voluntários da Pátria, 300</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>80440-020</t>
+          <t>80005-430</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>(41) 3340-5500</t>
-        </is>
-      </c>
-      <c r="K26" s="5" t="inlineStr">
-        <is>
-          <t>contato@clinicaartro.com.br</t>
-        </is>
-      </c>
-      <c r="L26" s="6" t="inlineStr"/>
-      <c r="M26" s="7" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="N26" s="8" t="inlineStr"/>
+          <t>(41) 3340-3030</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr"/>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="inlineStr"/>
+      <c r="N26" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2290,56 +2310,56 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>CLINICA LOS ANGELES</t>
+          <t>OFTALMO CURITIBA - HOSPITAL DA VISAO</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>02541094000131</t>
+          <t>80764889000112</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Anestesista, Angiologia, Buco Maxilo Facial, Cardiologia, Cirurgia da Mão, Cirurgia de Cabeça e Pescoço, Cirurgia do Aparelho Digestivo, Cirurgia Oncológica, Cirurgia Pediátrica, Cirurgia Plástica, Cirurgia Vascular, Cirurgias Ginecológica, Dermatologia, Infectologia, Ortopedia e Traumatologia, Otorrinolaringologia, Proctologia, Urologia</t>
+          <t>Oftalmologia</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Curitiba</t>
+          <t>São José dos Pinhais</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Batel</t>
+          <t>São Pedro</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>Avenida Sete de Setembro, 6520, Terreo</t>
+          <t>Rua Alcídio Viana, 1001, 5º andar consultório 53 exames sala 51e 52</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>80240-000</t>
+          <t>83005-560</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>(41) 3343-3103</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>loyolaodilon@gmail.com</t>
-        </is>
-      </c>
-      <c r="L27" s="6" t="inlineStr"/>
-      <c r="M27" s="7" t="inlineStr">
-        <is>
-          <t>✔</t>
-        </is>
-      </c>
-      <c r="N27" s="8" t="inlineStr"/>
+          <t>(41) 3146-1566</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr"/>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="inlineStr"/>
+      <c r="N27" s="8" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2354,17 +2374,17 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>CLINICA QUINTA DO SOL</t>
+          <t>ARTRO CLINICA ORTOPEDICA</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>78416393000106</t>
+          <t>11402669000126</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Psicologia, Psiquiatria</t>
+          <t>Ortopedia e Traumatologia</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -2374,27 +2394,27 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Jardim das Américas</t>
+          <t>Batel</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>Avenida Coronel Francisco Heráclito dos Santos, 1180</t>
+          <t>Avenida Vicente Machado, 2411</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>81530-001</t>
+          <t>80440-020</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>(41) 3267-6969</t>
+          <t>(41) 3340-5500</t>
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
         <is>
-          <t>convenios@clinicaquintadosol.com.br</t>
+          <t>contato@clinicaartro.com.br</t>
         </is>
       </c>
       <c r="L28" s="6" t="inlineStr"/>
@@ -2418,17 +2438,17 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL DE OLHOS DO PARANÁ</t>
+          <t>CLINICA LOS ANGELES</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>76104058000147</t>
+          <t>02541094000131</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>Oftalmologia</t>
+          <t>Anestesista, Angiologia, Buco Maxilo Facial, Cardiologia, Cirurgia da Mão, Cirurgia de Cabeça e Pescoço, Cirurgia do Aparelho Digestivo, Cirurgia Oncológica, Cirurgia Pediátrica, Cirurgia Plástica, Cirurgia Vascular, Cirurgias Ginecológica, Dermatologia, Infectologia, Ortopedia e Traumatologia, Otorrinolaringologia, Proctologia, Urologia</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
@@ -2443,22 +2463,22 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>Alameda Presidente Taunay, 483</t>
+          <t>Avenida Sete de Setembro, 6520, Terreo</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>80420-180</t>
+          <t>80240-000</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>(41) 3222-4222</t>
+          <t>(41) 3343-3103</t>
         </is>
       </c>
       <c r="K29" s="5" t="inlineStr">
         <is>
-          <t>comercial@hopr.com.br</t>
+          <t>loyolaodilon@gmail.com</t>
         </is>
       </c>
       <c r="L29" s="6" t="inlineStr"/>
@@ -2482,17 +2502,17 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL E MATERNIDADE NOSSA SENHORA DE FATIMA</t>
+          <t>CLINICA QUINTA DO SOL</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>75055772002920</t>
+          <t>78416393000106</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Análises Clínicas, Anatomia Patológica e Citopatologia, Clínica Geral, Ginecologia, Obstetrícia, Patologia Clínica/Medicina Laboratorial, Pediatria, Radiodiagnóstico, Ultrassonografia</t>
+          <t>Psicologia, Psiquiatria</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -2502,25 +2522,29 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Centro</t>
+          <t>Jardim das Américas</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>Avenida Visconde de Guarapuava, 3077</t>
+          <t>Avenida Coronel Francisco Heráclito dos Santos, 1180</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>80010-100</t>
+          <t>81530-001</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>(41) 3262-1212</t>
-        </is>
-      </c>
-      <c r="K30" s="5" t="inlineStr"/>
+          <t>(41) 3267-6969</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr">
+        <is>
+          <t>convenios@clinicaquintadosol.com.br</t>
+        </is>
+      </c>
       <c r="L30" s="6" t="inlineStr"/>
       <c r="M30" s="7" t="inlineStr">
         <is>
@@ -2542,17 +2566,17 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL ERASTINHO</t>
+          <t>HOSPITAL DE OLHOS DO PARANÁ</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>76591049000985</t>
+          <t>76104058000147</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Oncologia, Oncologia Pediatrica, Pediatria, Pronto Socorro Oncológico</t>
+          <t>Oftalmologia</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -2562,25 +2586,29 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Jardim das Américas</t>
+          <t>Batel</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Rua Doutor Ovande do Amaral, 201</t>
+          <t>Alameda Presidente Taunay, 483</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>81520-060</t>
+          <t>80420-180</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>(41) 3165-4504</t>
-        </is>
-      </c>
-      <c r="K31" s="5" t="inlineStr"/>
+          <t>(41) 3222-4222</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>comercial@hopr.com.br</t>
+        </is>
+      </c>
       <c r="L31" s="6" t="inlineStr"/>
       <c r="M31" s="7" t="inlineStr">
         <is>
@@ -2602,17 +2630,17 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL HEIDELBERG</t>
+          <t>HOSPITAL E MATERNIDADE NOSSA SENHORA DE FATIMA</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>76440577000186</t>
+          <t>75055772002920</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Psiquiatria</t>
+          <t>Análises Clínicas, Anatomia Patológica e Citopatologia, Clínica Geral, Ginecologia, Obstetrícia, Patologia Clínica/Medicina Laboratorial, Pediatria, Radiodiagnóstico, Ultrassonografia</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -2622,29 +2650,25 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Santa Felicidade</t>
+          <t>Centro</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>Rua Via Vêneto, 2000, Atendimento de consultas eletivas</t>
+          <t>Avenida Visconde de Guarapuava, 3077</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>82400-020</t>
+          <t>80010-100</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>(41) 3320-4940</t>
-        </is>
-      </c>
-      <c r="K32" s="5" t="inlineStr">
-        <is>
-          <t>faturamento@clinicaheidelberg.com.br</t>
-        </is>
-      </c>
+          <t>(41) 3262-1212</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr"/>
       <c r="L32" s="6" t="inlineStr"/>
       <c r="M32" s="7" t="inlineStr">
         <is>
@@ -2676,7 +2700,7 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Pronto Socorro Psquiatria, Psiquiatria</t>
+          <t>Psiquiatria</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -2686,22 +2710,22 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Mercês</t>
+          <t>Santa Felicidade</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>Rua Padre Agostinho, 687</t>
+          <t>Rua Via Vêneto, 2000, Atendimento de consultas eletivas</t>
         </is>
       </c>
       <c r="I33" s="5" t="inlineStr">
         <is>
-          <t>80430-050</t>
+          <t>82400-020</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>(41) 3320-4900</t>
+          <t>(41) 3320-4940</t>
         </is>
       </c>
       <c r="K33" s="5" t="inlineStr">
@@ -2730,17 +2754,17 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>HOSPITAL INFANTIL PEQUENO PRINCIPE</t>
+          <t>HOSPITAL HEIDELBERG</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>76591569000130</t>
+          <t>76440577000186</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Cirurgia Pediátrica, Dermatologia Pediátrica, Neurologia Pediátrica, Oncologia, Otorrinolaringologia, Pediatria, Pronto Socorro Pediatria, Reumatologia Infantil</t>
+          <t>Pronto Socorro Psquiatria, Psiquiatria</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -2750,25 +2774,29 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Água Verde</t>
+          <t>Mercês</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>Rua Desembargador Motta, 1070</t>
+          <t>Rua Padre Agostinho, 687</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr">
         <is>
-          <t>80250-060</t>
+          <t>80430-050</t>
         </is>
       </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>(41) 3310-1010</t>
-        </is>
-      </c>
-      <c r="K34" s="5" t="inlineStr"/>
+          <t>(41) 3320-4900</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr">
+        <is>
+          <t>faturamento@clinicaheidelberg.com.br</t>
+        </is>
+      </c>
       <c r="L34" s="6" t="inlineStr"/>
       <c r="M34" s="7" t="inlineStr">
         <is>
@@ -38147,7 +38175,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>461</v>
+        <v>464</v>
       </c>
     </row>
     <row r="7">
@@ -38177,7 +38205,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>230</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9"/>
@@ -38196,21 +38224,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>400 QP + 600 QC</t>
+          <t>400 QP + 600 QC + CIM QC</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>400 QP + 600 QC + CIM QC</t>
+          <t>400 QP + 600 QC</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13">
@@ -38220,7 +38248,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14">
@@ -38283,13 +38311,13 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C19" t="n">
         <v>16</v>
       </c>
       <c r="D19" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20">
@@ -38299,13 +38327,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C20" t="n">
         <v>21</v>
       </c>
       <c r="D20" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="21">
@@ -38482,13 +38510,13 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C32" t="n">
         <v>430</v>
       </c>
       <c r="D32" t="n">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="33">
@@ -38504,7 +38532,7 @@
         <v>45</v>
       </c>
       <c r="D33" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34">
@@ -38638,7 +38666,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Almirante Tamandaré</t>
+          <t>Tijucas do Sul</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -38654,7 +38682,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Quatro Barras</t>
+          <t>Almirante Tamandaré</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -38670,7 +38698,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tijucas do Sul</t>
+          <t>Quatro Barras</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -38686,7 +38714,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Itaperuçu</t>
+          <t>Mandirituba</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -38696,13 +38724,13 @@
         <v>1</v>
       </c>
       <c r="D45" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Lapa</t>
+          <t>Itaperuçu</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -38712,7 +38740,7 @@
         <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -38734,7 +38762,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Mandirituba</t>
+          <t>Lapa</t>
         </is>
       </c>
       <c r="B48" t="n">

</xml_diff>